<commit_message>
🔧 Halkbank POS düzeltme: Satış Toplamı ile birebir (2.639.707,37)
24/06'daki işlem tipi boş 300 TL'lik kayıt hariç tutuldu.
GÜNLÜK TOPLAM yerine kart tipi tanımlı satış detayları toplandı.
Sonuç PDF 'Satış Toplamı' 2.639.707,37 (3357 adet) ile birebir eşleşti.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISIK_PETROL-HALKBANK_POS-Gunluk_Brut-Haziran2026.xlsx
+++ b/ISIK_PETROL-HALKBANK_POS-Gunluk_Brut-Haziran2026.xlsx
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>32899.16</v>
+        <v>32599.16</v>
       </c>
     </row>
     <row r="26">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>2640007.37</v>
+        <v>2639707.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>